<commit_message>
fix: regenerate TestCase_TravelApp.xlsx with correct content
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestCase_TravelApp.xlsx
+++ b/TestCase_TravelApp.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Tổng hợp" sheetId="1" r:id="rId1"/>
-    <sheet name="Chi tiết Test Case" sheetId="2" r:id="rId2"/>
+    <sheet name="Tong hop" sheetId="1" r:id="rId1"/>
+    <sheet name="Chi tiet Test Case" sheetId="2" r:id="rId2"/>
     <sheet name="API Test Results" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,125 +399,233 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>BÁO CÁO KẾT QUẢ KIỂM THỬ - TRAVEL APP</v>
       </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Dự án:</v>
+        <v>Dự án</v>
       </c>
       <c r="B3" t="str">
         <v>Travel App (Flutter)</v>
       </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Người kiểm thử:</v>
+        <v>Người kiểm thử</v>
       </c>
       <c r="B4" t="str">
         <v>SangIT465</v>
       </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ngày kiểm thử:</v>
+        <v>Ngày kiểm thử</v>
       </c>
       <c r="B5" t="str">
         <v>14/05/2026</v>
       </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Base URL:</v>
+        <v>Base URL</v>
       </c>
       <c r="B6" t="str">
         <v>http://localhost:3000/api</v>
       </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Tổng số test case:</v>
-      </c>
-      <c r="B8">
-        <v>33</v>
+        <v>THỐNG KÊ TỔNG QUAN</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PASS:</v>
+        <v>Tổng test case</v>
       </c>
       <c r="B9">
         <v>33</v>
       </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>FAIL:</v>
+        <v>PASS</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>33</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Tỷ lệ Pass:</v>
-      </c>
-      <c r="B11" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Tỷ lệ Pass</v>
+      </c>
+      <c r="B12" t="str">
         <v>100%</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Phân loại theo Module:</v>
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Module</v>
+        <v>THỐNG KÊ THEO MODULE</v>
       </c>
       <c r="B14" t="str">
-        <v>Tổng TC</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>PASS</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>FAIL</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Authentication</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-      <c r="C15">
-        <v>5</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
+        <v>Module</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tổng TC</v>
+      </c>
+      <c r="C15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="D15" t="str">
+        <v>FAIL</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>API - Explore</v>
+        <v>Authentication</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -525,13 +633,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>API - Tours</v>
+        <v>API - Explore</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -539,13 +647,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>API - My Trips</v>
+        <v>API - Tours</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -553,13 +661,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>API - Next Trips</v>
+        <v>API - My Trips</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -567,7 +675,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>API - Past Trips</v>
+        <v>API - Next Trips</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -581,13 +689,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>API - Payment</v>
+        <v>API - Past Trips</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -595,13 +703,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>API - Profile</v>
+        <v>API - Payment</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -609,13 +717,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>API - TourMore</v>
+        <v>API - Profile</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -623,13 +731,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>API - WishList</v>
+        <v>API - TourMore</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -637,13 +745,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>API - News</v>
+        <v>API - WishList</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -651,7 +759,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>API - Guides</v>
+        <v>API - News</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -665,7 +773,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>UI - Home</v>
+        <v>API - Guides</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -679,7 +787,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>UI - Explore</v>
+        <v>UI - Home</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -693,7 +801,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>UI - TourMore</v>
+        <v>UI - Explore</v>
       </c>
       <c r="B29">
         <v>1</v>
@@ -707,7 +815,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>UI - Payment</v>
+        <v>UI - TourMore</v>
       </c>
       <c r="B30">
         <v>1</v>
@@ -721,7 +829,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>UI - WishList</v>
+        <v>UI - Payment</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -733,28 +841,41 @@
         <v>0</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>UI - WishList</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:J34"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="32.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
     <col min="8" max="8" width="35.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -788,11 +909,8 @@
       <c r="J1" t="str">
         <v>Trạng thái</v>
       </c>
-      <c r="K1" t="str">
-        <v>Ghi chú</v>
-      </c>
-    </row>
-    <row r="2" xml:space="preserve">
+    </row>
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -806,17 +924,13 @@
         <v>Đăng nhập thành công</v>
       </c>
       <c r="E2" t="str">
-        <v>Người dùng nhập đúng email và password</v>
-      </c>
-      <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở app
-2. Nhập email hợp lệ
-3. Nhập password đúng
-4. Nhấn Đăng nhập</v>
-      </c>
-      <c r="G2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Email: test@gmail.com
-Password: 123456</v>
+        <v>Nhập đúng email và password</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1. Mở app 2. Nhập email hợp lệ 3. Nhập password đúng 4. Nhấn Đăng nhập</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Email: test@gmail.com / Password: 123456</v>
       </c>
       <c r="H2" t="str">
         <v>Chuyển đến màn hình Home</v>
@@ -827,11 +941,8 @@
       <c r="J2" t="str">
         <v>PASS</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
+    </row>
+    <row r="3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -845,17 +956,13 @@
         <v>Đăng nhập sai password</v>
       </c>
       <c r="E3" t="str">
-        <v>Người dùng nhập sai password</v>
-      </c>
-      <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở app
-2. Nhập email hợp lệ
-3. Nhập password sai
-4. Nhấn Đăng nhập</v>
-      </c>
-      <c r="G3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Email: test@gmail.com
-Password: saipass</v>
+        <v>Nhập sai password</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1. Mở app 2. Nhập email hợp lệ 3. Nhập password sai 4. Nhấn Đăng nhập</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Email: test@gmail.com / Password: saipass</v>
       </c>
       <c r="H3" t="str">
         <v>Hiển thị thông báo lỗi</v>
@@ -866,11 +973,8 @@
       <c r="J3" t="str">
         <v>PASS</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
+    </row>
+    <row r="4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -884,32 +988,25 @@
         <v>Đăng nhập email trống</v>
       </c>
       <c r="E4" t="str">
-        <v>Người dùng để trống email</v>
-      </c>
-      <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở app
-2. Để trống email
-3. Nhập password
-4. Nhấn Đăng nhập</v>
-      </c>
-      <c r="G4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Email: (trống)
-Password: 123456</v>
+        <v>Để trống email</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1. Mở app 2. Để trống email 3. Nhập password 4. Nhấn Đăng nhập</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Email: (trống) / Password: 123456</v>
       </c>
       <c r="H4" t="str">
-        <v>Hiển thị thông báo yêu cầu nhập email</v>
+        <v>Yêu cầu nhập email</v>
       </c>
       <c r="I4" t="str">
-        <v>Hiển thị thông báo yêu cầu nhập email</v>
+        <v>Yêu cầu nhập email</v>
       </c>
       <c r="J4" t="str">
         <v>PASS</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
+    </row>
+    <row r="5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -923,17 +1020,13 @@
         <v>Đăng ký tài khoản mới</v>
       </c>
       <c r="E5" t="str">
-        <v>Người dùng tạo tài khoản mới thành công</v>
-      </c>
-      <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở app
-2. Nhấn Đăng ký
-3. Điền đầy đủ thông tin
-4. Nhấn Xác nhận</v>
-      </c>
-      <c r="G5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Email: newuser@gmail.com
-Password: 123456</v>
+        <v>Tạo tài khoản mới thành công</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1. Nhấn Đăng ký 2. Điền đầy đủ thông tin 3. Nhấn Xác nhận</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Email: newuser@gmail.com / Password: 123456</v>
       </c>
       <c r="H5" t="str">
         <v>Tài khoản được tạo thành công</v>
@@ -944,11 +1037,8 @@
       <c r="J5" t="str">
         <v>PASS</v>
       </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+    </row>
+    <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -964,25 +1054,20 @@
       <c r="E6" t="str">
         <v>Gửi email đặt lại mật khẩu</v>
       </c>
-      <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Nhấn Quên mật khẩu
-2. Nhập email
-3. Nhấn Gửi</v>
+      <c r="F6" t="str">
+        <v>1. Nhấn Quên mật khẩu 2. Nhập email 3. Nhấn Gửi</v>
       </c>
       <c r="G6" t="str">
         <v>Email: test@gmail.com</v>
       </c>
       <c r="H6" t="str">
-        <v>Email đặt lại được gửi thành công</v>
+        <v>Email đặt lại được gửi</v>
       </c>
       <c r="I6" t="str">
-        <v>Email đặt lại được gửi thành công</v>
+        <v>Email đặt lại được gửi</v>
       </c>
       <c r="J6" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K6" t="str">
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -1002,22 +1087,19 @@
         <v>Lấy dữ liệu trang khám phá</v>
       </c>
       <c r="F7" t="str">
-        <v>Gửi GET request đến /api/explore</v>
+        <v>Gửi GET /api/explore</v>
       </c>
       <c r="G7" t="str">
         <v>Không có</v>
       </c>
       <c r="H7" t="str">
-        <v>Status 200, trả về banners, tours, guides, news</v>
+        <v>200 - banners, tours, guides, news</v>
       </c>
       <c r="I7" t="str">
-        <v>Status 200, trả về đúng dữ liệu</v>
+        <v>200 - trả về đúng dữ liệu</v>
       </c>
       <c r="J7" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K7" t="str">
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -1037,22 +1119,19 @@
         <v>Toggle like tour</v>
       </c>
       <c r="F8" t="str">
-        <v>Gửi PATCH request đến /api/tours/1/like</v>
+        <v>Gửi PATCH /api/tours/1/like</v>
       </c>
       <c r="G8" t="str">
         <v>id: 1</v>
       </c>
       <c r="H8" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="I8" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="J8" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K8" t="str">
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -1072,22 +1151,19 @@
         <v>Toggle lưu tour</v>
       </c>
       <c r="F9" t="str">
-        <v>Gửi PATCH request đến /api/tours/1/save</v>
+        <v>Gửi PATCH /api/tours/1/save</v>
       </c>
       <c r="G9" t="str">
         <v>id: 1</v>
       </c>
       <c r="H9" t="str">
-        <v>Status 200, saved đảo ngược</v>
+        <v>200 - saved đảo ngược</v>
       </c>
       <c r="I9" t="str">
-        <v>Status 200, saved đảo ngược</v>
+        <v>200 - saved đảo ngược</v>
       </c>
       <c r="J9" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K9" t="str">
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -1107,22 +1183,19 @@
         <v>Lấy danh sách chuyến đi hiện tại</v>
       </c>
       <c r="F10" t="str">
-        <v>Gửi GET request đến /api/my-trips/current</v>
+        <v>Gửi GET /api/my-trips/current</v>
       </c>
       <c r="G10" t="str">
         <v>Không có</v>
       </c>
       <c r="H10" t="str">
-        <v>Status 200, danh sách chuyến đi</v>
+        <v>200 - danh sách chuyến đi</v>
       </c>
       <c r="I10" t="str">
-        <v>Status 200, trả về 3 chuyến đi</v>
+        <v>200 - trả về 3 chuyến đi</v>
       </c>
       <c r="J10" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K10" t="str">
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -1136,28 +1209,25 @@
         <v>TC_API_05</v>
       </c>
       <c r="D11" t="str">
-        <v>GET /api/my-trips/detail/:id</v>
+        <v>GET /api/my-trips/detail/1</v>
       </c>
       <c r="E11" t="str">
-        <v>Lấy chi tiết chuyến đi hiện tại</v>
+        <v>Chi tiết chuyến đi hiện tại</v>
       </c>
       <c r="F11" t="str">
-        <v>Gửi GET request đến /api/my-trips/detail/1</v>
+        <v>Gửi GET /api/my-trips/detail/1</v>
       </c>
       <c r="G11" t="str">
         <v>id: 1</v>
       </c>
       <c r="H11" t="str">
-        <v>Status 200, thông tin chi tiết chuyến đi</v>
+        <v>200 - chi tiết chuyến đi</v>
       </c>
       <c r="I11" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="J11" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K11" t="str">
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -1171,28 +1241,25 @@
         <v>TC_API_06</v>
       </c>
       <c r="D12" t="str">
-        <v>GET /api/my-trips/detail/:id (not found)</v>
+        <v>GET /api/my-trips/detail/999</v>
       </c>
       <c r="E12" t="str">
-        <v>ID không tồn tại</v>
+        <v>ID chuyến đi không tồn tại</v>
       </c>
       <c r="F12" t="str">
-        <v>Gửi GET request đến /api/my-trips/detail/999</v>
+        <v>Gửi GET /api/my-trips/detail/999</v>
       </c>
       <c r="G12" t="str">
         <v>id: 999</v>
       </c>
       <c r="H12" t="str">
-        <v>Status 404, message: Trip detail not found</v>
+        <v>404 - Trip detail not found</v>
       </c>
       <c r="I12" t="str">
-        <v>Status 404, trả về đúng message</v>
+        <v>404 - đúng message</v>
       </c>
       <c r="J12" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K12" t="str">
-        <v/>
       </c>
     </row>
     <row r="13">
@@ -1212,22 +1279,19 @@
         <v>Lấy danh sách chuyến đi sắp tới</v>
       </c>
       <c r="F13" t="str">
-        <v>Gửi GET request đến /api/next-trips</v>
+        <v>Gửi GET /api/next-trips</v>
       </c>
       <c r="G13" t="str">
         <v>Không có</v>
       </c>
       <c r="H13" t="str">
-        <v>Status 200, danh sách chuyến đi</v>
+        <v>200 - danh sách chuyến đi</v>
       </c>
       <c r="I13" t="str">
-        <v>Status 200, trả về 3 chuyến đi</v>
+        <v>200 - trả về 3 chuyến đi</v>
       </c>
       <c r="J13" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K13" t="str">
-        <v/>
       </c>
     </row>
     <row r="14">
@@ -1241,28 +1305,25 @@
         <v>TC_API_08</v>
       </c>
       <c r="D14" t="str">
-        <v>GET /api/next-trips/detail/:id</v>
+        <v>GET /api/next-trips/detail/1</v>
       </c>
       <c r="E14" t="str">
-        <v>Lấy chi tiết chuyến đi sắp tới</v>
+        <v>Chi tiết chuyến đi sắp tới</v>
       </c>
       <c r="F14" t="str">
-        <v>Gửi GET request đến /api/next-trips/detail/1</v>
+        <v>Gửi GET /api/next-trips/detail/1</v>
       </c>
       <c r="G14" t="str">
         <v>id: 1</v>
       </c>
       <c r="H14" t="str">
-        <v>Status 200, thông tin chi tiết</v>
+        <v>200 - chi tiết</v>
       </c>
       <c r="I14" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="J14" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K14" t="str">
-        <v/>
       </c>
     </row>
     <row r="15">
@@ -1282,22 +1343,19 @@
         <v>Lấy danh sách chuyến đi đã qua</v>
       </c>
       <c r="F15" t="str">
-        <v>Gửi GET request đến /api/past-trips</v>
+        <v>Gửi GET /api/past-trips</v>
       </c>
       <c r="G15" t="str">
         <v>Không có</v>
       </c>
       <c r="H15" t="str">
-        <v>Status 200, danh sách chuyến đi</v>
+        <v>200 - danh sách chuyến đi</v>
       </c>
       <c r="I15" t="str">
-        <v>Status 200, trả về 2 chuyến đi</v>
+        <v>200 - trả về 2 chuyến đi</v>
       </c>
       <c r="J15" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K15" t="str">
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -1311,28 +1369,25 @@
         <v>TC_API_10</v>
       </c>
       <c r="D16" t="str">
-        <v>GET /api/past-trips/detail/:id</v>
+        <v>GET /api/past-trips/detail/201</v>
       </c>
       <c r="E16" t="str">
-        <v>Lấy chi tiết chuyến đi đã qua</v>
+        <v>Chi tiết chuyến đi đã qua</v>
       </c>
       <c r="F16" t="str">
-        <v>Gửi GET request đến /api/past-trips/detail/201</v>
+        <v>Gửi GET /api/past-trips/detail/201</v>
       </c>
       <c r="G16" t="str">
         <v>id: 201</v>
       </c>
       <c r="H16" t="str">
-        <v>Status 200, thông tin chi tiết</v>
+        <v>200 - chi tiết</v>
       </c>
       <c r="I16" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="J16" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K16" t="str">
-        <v/>
       </c>
     </row>
     <row r="17">
@@ -1352,22 +1407,19 @@
         <v>Xem trước thông tin thanh toán</v>
       </c>
       <c r="F17" t="str">
-        <v>Gửi GET request đến /api/payment/preview</v>
+        <v>Gửi GET /api/payment/preview</v>
       </c>
       <c r="G17" t="str">
         <v>Không có</v>
       </c>
       <c r="H17" t="str">
-        <v>Status 200, thông tin thanh toán</v>
+        <v>200 - thông tin thanh toán</v>
       </c>
       <c r="I17" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="J17" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K17" t="str">
-        <v/>
       </c>
     </row>
     <row r="18">
@@ -1387,22 +1439,19 @@
         <v>Xử lý thanh toán thành công</v>
       </c>
       <c r="F18" t="str">
-        <v>Gửi POST request đến /api/payment/process với body</v>
+        <v>Gửi POST /api/payment/process với body</v>
       </c>
       <c r="G18" t="str">
-        <v>travelers: 2, total: 20</v>
+        <v>travelers: 2 / total: 20</v>
       </c>
       <c r="H18" t="str">
-        <v>Status 200, success: true</v>
+        <v>200 - success: true</v>
       </c>
       <c r="I18" t="str">
-        <v>Status 200, success: true</v>
+        <v>200 - success: true</v>
       </c>
       <c r="J18" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K18" t="str">
-        <v/>
       </c>
     </row>
     <row r="19">
@@ -1416,28 +1465,25 @@
         <v>TC_API_13</v>
       </c>
       <c r="D19" t="str">
-        <v>POST /api/payment/process (thiếu body)</v>
+        <v>POST /api/payment/process (body rỗng)</v>
       </c>
       <c r="E19" t="str">
-        <v>Xử lý thanh toán với body rỗng</v>
+        <v>Thanh toán không có body</v>
       </c>
       <c r="F19" t="str">
-        <v>Gửi POST request đến /api/payment/process không có body</v>
+        <v>Gửi POST /api/payment/process không có body</v>
       </c>
       <c r="G19" t="str">
         <v>(trống)</v>
       </c>
       <c r="H19" t="str">
-        <v>Status 200, dùng giá trị mặc định</v>
+        <v>200 - dùng giá trị mặc định</v>
       </c>
       <c r="I19" t="str">
-        <v>Status 200, dùng giá trị mặc định</v>
+        <v>200 - dùng giá trị mặc định</v>
       </c>
       <c r="J19" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K19" t="str">
-        <v/>
       </c>
     </row>
     <row r="20">
@@ -1457,22 +1503,19 @@
         <v>Lấy hồ sơ người dùng</v>
       </c>
       <c r="F20" t="str">
-        <v>Gửi GET request đến /api/profile</v>
+        <v>Gửi GET /api/profile</v>
       </c>
       <c r="G20" t="str">
         <v>Không có</v>
       </c>
       <c r="H20" t="str">
-        <v>Status 200, thông tin profile, photos, journeys</v>
+        <v>200 - profile, photos, journeys</v>
       </c>
       <c r="I20" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="J20" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K20" t="str">
-        <v/>
       </c>
     </row>
     <row r="21">
@@ -1492,22 +1535,19 @@
         <v>Lấy danh sách tour</v>
       </c>
       <c r="F21" t="str">
-        <v>Gửi GET request đến /api/tourMore</v>
+        <v>Gửi GET /api/tourMore</v>
       </c>
       <c r="G21" t="str">
         <v>Không có</v>
       </c>
       <c r="H21" t="str">
-        <v>Status 200, danh sách 8 tour</v>
+        <v>200 - danh sách 8 tour</v>
       </c>
       <c r="I21" t="str">
-        <v>Status 200, trả về 8 tour</v>
+        <v>200 - trả về 8 tour</v>
       </c>
       <c r="J21" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K21" t="str">
-        <v/>
       </c>
     </row>
     <row r="22">
@@ -1527,22 +1567,19 @@
         <v>Tìm kiếm tour theo từ khóa</v>
       </c>
       <c r="F22" t="str">
-        <v>Gửi GET request đến /api/tourMore?q=hanoi</v>
+        <v>Gửi GET /api/tourMore?q=hanoi</v>
       </c>
       <c r="G22" t="str">
         <v>q: hanoi</v>
       </c>
       <c r="H22" t="str">
-        <v>Status 200, kết quả lọc theo từ khóa</v>
+        <v>200 - kết quả lọc</v>
       </c>
       <c r="I22" t="str">
-        <v>Status 200, trả về tour có 'hanoi'</v>
+        <v>200 - tour có hanoi</v>
       </c>
       <c r="J22" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K22" t="str">
-        <v/>
       </c>
     </row>
     <row r="23">
@@ -1556,28 +1593,25 @@
         <v>TC_API_17</v>
       </c>
       <c r="D23" t="str">
-        <v>PATCH /api/tourMore/tours/:id/favorite</v>
+        <v>PATCH /api/tourMore/tours/1/favorite</v>
       </c>
       <c r="E23" t="str">
         <v>Toggle yêu thích tour</v>
       </c>
       <c r="F23" t="str">
-        <v>Gửi PATCH request đến /api/tourMore/tours/1/favorite</v>
+        <v>Gửi PATCH /api/tourMore/tours/1/favorite</v>
       </c>
       <c r="G23" t="str">
         <v>id: 1</v>
       </c>
       <c r="H23" t="str">
-        <v>Status 200, favorite đảo ngược</v>
+        <v>200 - favorite đảo ngược</v>
       </c>
       <c r="I23" t="str">
-        <v>Status 200, favorite đảo ngược</v>
+        <v>200 - favorite đảo ngược</v>
       </c>
       <c r="J23" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K23" t="str">
-        <v/>
       </c>
     </row>
     <row r="24">
@@ -1597,22 +1631,19 @@
         <v>Lấy danh sách yêu thích</v>
       </c>
       <c r="F24" t="str">
-        <v>Gửi GET request đến /api/wish-list</v>
+        <v>Gửi GET /api/wish-list</v>
       </c>
       <c r="G24" t="str">
         <v>Không có</v>
       </c>
       <c r="H24" t="str">
-        <v>Status 200, danh sách wish list</v>
+        <v>200 - danh sách wish list</v>
       </c>
       <c r="I24" t="str">
-        <v>Status 200, trả về 2 tour</v>
+        <v>200 - trả về 2 tour</v>
       </c>
       <c r="J24" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K24" t="str">
-        <v/>
       </c>
     </row>
     <row r="25">
@@ -1626,28 +1657,25 @@
         <v>TC_API_19</v>
       </c>
       <c r="D25" t="str">
-        <v>PATCH /api/wish-list/:id/like</v>
+        <v>PATCH /api/wish-list/301/like</v>
       </c>
       <c r="E25" t="str">
         <v>Toggle like trong wish list</v>
       </c>
       <c r="F25" t="str">
-        <v>Gửi PATCH request đến /api/wish-list/301/like</v>
+        <v>Gửi PATCH /api/wish-list/301/like</v>
       </c>
       <c r="G25" t="str">
         <v>id: 301</v>
       </c>
       <c r="H25" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="I25" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="J25" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K25" t="str">
-        <v/>
       </c>
     </row>
     <row r="26">
@@ -1661,28 +1689,25 @@
         <v>TC_API_20</v>
       </c>
       <c r="D26" t="str">
-        <v>DELETE /api/wish-list/:id</v>
+        <v>DELETE /api/wish-list/302</v>
       </c>
       <c r="E26" t="str">
         <v>Xóa tour khỏi wish list</v>
       </c>
       <c r="F26" t="str">
-        <v>Gửi DELETE request đến /api/wish-list/302</v>
+        <v>Gửi DELETE /api/wish-list/302</v>
       </c>
       <c r="G26" t="str">
         <v>id: 302</v>
       </c>
       <c r="H26" t="str">
-        <v>Status 200, xóa thành công</v>
+        <v>200 - xóa thành công</v>
       </c>
       <c r="I26" t="str">
-        <v>Status 200, xóa thành công</v>
+        <v>200 - xóa thành công</v>
       </c>
       <c r="J26" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K26" t="str">
-        <v/>
       </c>
     </row>
     <row r="27">
@@ -1696,28 +1721,25 @@
         <v>TC_API_21</v>
       </c>
       <c r="D27" t="str">
-        <v>DELETE /api/wish-list/:id (not found)</v>
+        <v>DELETE /api/wish-list/999</v>
       </c>
       <c r="E27" t="str">
         <v>Xóa tour không tồn tại</v>
       </c>
       <c r="F27" t="str">
-        <v>Gửi DELETE request đến /api/wish-list/999</v>
+        <v>Gửi DELETE /api/wish-list/999</v>
       </c>
       <c r="G27" t="str">
         <v>id: 999</v>
       </c>
       <c r="H27" t="str">
-        <v>Status 404, message: Trip not found</v>
+        <v>404 - Trip not found</v>
       </c>
       <c r="I27" t="str">
-        <v>Status 404, trả về đúng message</v>
+        <v>404 - đúng message</v>
       </c>
       <c r="J27" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K27" t="str">
-        <v/>
       </c>
     </row>
     <row r="28">
@@ -1737,22 +1759,19 @@
         <v>Lấy danh sách tin tức</v>
       </c>
       <c r="F28" t="str">
-        <v>Gửi GET request đến /api/news</v>
+        <v>Gửi GET /api/news</v>
       </c>
       <c r="G28" t="str">
         <v>Không có</v>
       </c>
       <c r="H28" t="str">
-        <v>Status 200, danh sách tin tức</v>
+        <v>200 - danh sách tin tức</v>
       </c>
       <c r="I28" t="str">
-        <v>Status 200, trả về 3 tin tức</v>
+        <v>200 - trả về 3 tin tức</v>
       </c>
       <c r="J28" t="str">
         <v>PASS</v>
-      </c>
-      <c r="K28" t="str">
-        <v/>
       </c>
     </row>
     <row r="29">
@@ -1772,25 +1791,22 @@
         <v>Lấy danh sách hướng dẫn viên</v>
       </c>
       <c r="F29" t="str">
-        <v>Gửi GET request đến /api/guides</v>
+        <v>Gửi GET /api/guides</v>
       </c>
       <c r="G29" t="str">
         <v>Không có</v>
       </c>
       <c r="H29" t="str">
-        <v>Status 200, danh sách hướng dẫn viên</v>
+        <v>200 - danh sách hướng dẫn viên</v>
       </c>
       <c r="I29" t="str">
-        <v>Status 200, trả về 2 hướng dẫn viên</v>
+        <v>200 - trả về 2 hướng dẫn viên</v>
       </c>
       <c r="J29" t="str">
         <v>PASS</v>
       </c>
-      <c r="K29" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="30" xml:space="preserve">
+    </row>
+    <row r="30">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1801,20 +1817,19 @@
         <v>TC_UI_01</v>
       </c>
       <c r="D30" t="str">
-        <v>Hiển thị trang chủ</v>
+        <v>Hiển thị trang chủ đầy đủ</v>
       </c>
       <c r="E30" t="str">
         <v>Trang chủ load đầy đủ dữ liệu</v>
       </c>
-      <c r="F30" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Đăng nhập
-2. Quan sát màn hình Home</v>
+      <c r="F30" t="str">
+        <v>1. Đăng nhập 2. Quan sát màn hình Home</v>
       </c>
       <c r="G30" t="str">
         <v>Không có</v>
       </c>
       <c r="H30" t="str">
-        <v>Hiển thị banner, tour, hướng dẫn viên, tin tức</v>
+        <v>Banner, tour, hướng dẫn viên, tin tức</v>
       </c>
       <c r="I30" t="str">
         <v>Hiển thị đầy đủ</v>
@@ -1822,11 +1837,8 @@
       <c r="J30" t="str">
         <v>PASS</v>
       </c>
-      <c r="K30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31" xml:space="preserve">
+    </row>
+    <row r="31">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1837,14 +1849,13 @@
         <v>TC_UI_02</v>
       </c>
       <c r="D31" t="str">
-        <v>Like tour trên Explore</v>
+        <v>Like tour trên màn hình Explore</v>
       </c>
       <c r="E31" t="str">
-        <v>Người dùng like một tour</v>
-      </c>
-      <c r="F31" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Vào Explore
-2. Nhấn nút like trên tour</v>
+        <v>Nhấn like trên một tour</v>
+      </c>
+      <c r="F31" t="str">
+        <v>1. Vào Explore 2. Nhấn nút like trên tour</v>
       </c>
       <c r="G31" t="str">
         <v>Không có</v>
@@ -1858,11 +1869,8 @@
       <c r="J31" t="str">
         <v>PASS</v>
       </c>
-      <c r="K31" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="32" xml:space="preserve">
+    </row>
+    <row r="32">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1873,20 +1881,19 @@
         <v>TC_UI_03</v>
       </c>
       <c r="D32" t="str">
-        <v>Tìm kiếm tour</v>
+        <v>Tìm kiếm tour theo từ khóa</v>
       </c>
       <c r="E32" t="str">
-        <v>Người dùng nhập từ khóa tìm kiếm</v>
-      </c>
-      <c r="F32" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Vào Tour More
-2. Nhập từ khóa vào ô tìm kiếm</v>
+        <v>Nhập từ khóa vào ô tìm kiếm</v>
+      </c>
+      <c r="F32" t="str">
+        <v>1. Vào Tour More 2. Nhập từ khóa</v>
       </c>
       <c r="G32" t="str">
         <v>Từ khóa: hanoi</v>
       </c>
       <c r="H32" t="str">
-        <v>Hiển thị kết quả lọc theo từ khóa</v>
+        <v>Kết quả lọc theo từ khóa</v>
       </c>
       <c r="I32" t="str">
         <v>Hiển thị đúng kết quả</v>
@@ -1894,11 +1901,8 @@
       <c r="J32" t="str">
         <v>PASS</v>
       </c>
-      <c r="K32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33" xml:space="preserve">
+    </row>
+    <row r="33">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1909,21 +1913,19 @@
         <v>TC_UI_04</v>
       </c>
       <c r="D33" t="str">
-        <v>Xem trước thanh toán</v>
+        <v>Xem trước thông tin thanh toán</v>
       </c>
       <c r="E33" t="str">
-        <v>Màn hình thanh toán hiển thị đúng thông tin</v>
-      </c>
-      <c r="F33" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Chọn tour
-2. Nhấn Pay
-3. Xem màn hình Payment</v>
+        <v>Màn hình thanh toán hiển thị đúng</v>
+      </c>
+      <c r="F33" t="str">
+        <v>1. Chọn tour 2. Nhấn Pay 3. Xem Payment</v>
       </c>
       <c r="G33" t="str">
         <v>Không có</v>
       </c>
       <c r="H33" t="str">
-        <v>Hiển thị đúng thông tin tour, giá, số khách</v>
+        <v>Thông tin tour, giá, số khách đúng</v>
       </c>
       <c r="I33" t="str">
         <v>Hiển thị đúng</v>
@@ -1931,11 +1933,8 @@
       <c r="J33" t="str">
         <v>PASS</v>
       </c>
-      <c r="K33" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="34" xml:space="preserve">
+    </row>
+    <row r="34">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1949,11 +1948,10 @@
         <v>Xóa tour khỏi Wish List</v>
       </c>
       <c r="E34" t="str">
-        <v>Người dùng xóa tour khỏi danh sách yêu thích</v>
-      </c>
-      <c r="F34" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Vào Wish List
-2. Nhấn xóa tour</v>
+        <v>Nhấn xóa tour khỏi danh sách yêu thích</v>
+      </c>
+      <c r="F34" t="str">
+        <v>1. Vào Wish List 2. Nhấn xóa tour</v>
       </c>
       <c r="G34" t="str">
         <v>Không có</v>
@@ -1967,13 +1965,10 @@
       <c r="J34" t="str">
         <v>PASS</v>
       </c>
-      <c r="K34" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1983,8 +1978,8 @@
   <dimension ref="A1:G24"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="35.83203125" customWidth="1"/>
@@ -1996,10 +1991,10 @@
         <v>STT</v>
       </c>
       <c r="B1" t="str">
+        <v>Method</v>
+      </c>
+      <c r="C1" t="str">
         <v>Endpoint</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Method</v>
       </c>
       <c r="D1" t="str">
         <v>Dữ liệu Test</v>
@@ -2008,7 +2003,7 @@
         <v>Status Code</v>
       </c>
       <c r="F1" t="str">
-        <v>Kết quả</v>
+        <v>Kết quả thực tế</v>
       </c>
       <c r="G1" t="str">
         <v>Trạng thái</v>
@@ -2019,10 +2014,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C2" t="str">
         <v>/api/explore</v>
-      </c>
-      <c r="C2" t="str">
-        <v>GET</v>
       </c>
       <c r="D2" t="str">
         <v>Không có</v>
@@ -2031,7 +2026,7 @@
         <v>200</v>
       </c>
       <c r="F2" t="str">
-        <v>Status 200, trả về đúng dữ liệu</v>
+        <v>200 - trả về đúng dữ liệu</v>
       </c>
       <c r="G2" t="str">
         <v>PASS</v>
@@ -2042,10 +2037,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
+        <v>PATCH</v>
+      </c>
+      <c r="C3" t="str">
         <v>/api/tours/:id/like</v>
-      </c>
-      <c r="C3" t="str">
-        <v>PATCH</v>
       </c>
       <c r="D3" t="str">
         <v>id: 1</v>
@@ -2054,7 +2049,7 @@
         <v>200</v>
       </c>
       <c r="F3" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="G3" t="str">
         <v>PASS</v>
@@ -2065,10 +2060,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
+        <v>PATCH</v>
+      </c>
+      <c r="C4" t="str">
         <v>/api/tours/:id/save</v>
-      </c>
-      <c r="C4" t="str">
-        <v>PATCH</v>
       </c>
       <c r="D4" t="str">
         <v>id: 1</v>
@@ -2077,7 +2072,7 @@
         <v>200</v>
       </c>
       <c r="F4" t="str">
-        <v>Status 200, saved đảo ngược</v>
+        <v>200 - saved đảo ngược</v>
       </c>
       <c r="G4" t="str">
         <v>PASS</v>
@@ -2088,10 +2083,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C5" t="str">
         <v>/api/my-trips/current</v>
-      </c>
-      <c r="C5" t="str">
-        <v>GET</v>
       </c>
       <c r="D5" t="str">
         <v>Không có</v>
@@ -2100,7 +2095,7 @@
         <v>200</v>
       </c>
       <c r="F5" t="str">
-        <v>Status 200, trả về 3 chuyến đi</v>
+        <v>200 - trả về 3 chuyến đi</v>
       </c>
       <c r="G5" t="str">
         <v>PASS</v>
@@ -2111,10 +2106,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>/api/my-trips/detail/:id</v>
+        <v>GET</v>
       </c>
       <c r="C6" t="str">
-        <v>GET</v>
+        <v>/api/my-trips/detail/1</v>
       </c>
       <c r="D6" t="str">
         <v>id: 1</v>
@@ -2123,7 +2118,7 @@
         <v>200</v>
       </c>
       <c r="F6" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="G6" t="str">
         <v>PASS</v>
@@ -2134,10 +2129,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>/api/my-trips/detail/:id (not found)</v>
+        <v>GET</v>
       </c>
       <c r="C7" t="str">
-        <v>GET</v>
+        <v>/api/my-trips/detail/999</v>
       </c>
       <c r="D7" t="str">
         <v>id: 999</v>
@@ -2146,7 +2141,7 @@
         <v>200</v>
       </c>
       <c r="F7" t="str">
-        <v>Status 404, trả về đúng message</v>
+        <v>404 - đúng message</v>
       </c>
       <c r="G7" t="str">
         <v>PASS</v>
@@ -2157,10 +2152,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C8" t="str">
         <v>/api/next-trips</v>
-      </c>
-      <c r="C8" t="str">
-        <v>GET</v>
       </c>
       <c r="D8" t="str">
         <v>Không có</v>
@@ -2169,7 +2164,7 @@
         <v>200</v>
       </c>
       <c r="F8" t="str">
-        <v>Status 200, trả về 3 chuyến đi</v>
+        <v>200 - trả về 3 chuyến đi</v>
       </c>
       <c r="G8" t="str">
         <v>PASS</v>
@@ -2180,10 +2175,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>/api/next-trips/detail/:id</v>
+        <v>GET</v>
       </c>
       <c r="C9" t="str">
-        <v>GET</v>
+        <v>/api/next-trips/detail/1</v>
       </c>
       <c r="D9" t="str">
         <v>id: 1</v>
@@ -2192,7 +2187,7 @@
         <v>200</v>
       </c>
       <c r="F9" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="G9" t="str">
         <v>PASS</v>
@@ -2203,10 +2198,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C10" t="str">
         <v>/api/past-trips</v>
-      </c>
-      <c r="C10" t="str">
-        <v>GET</v>
       </c>
       <c r="D10" t="str">
         <v>Không có</v>
@@ -2215,7 +2210,7 @@
         <v>200</v>
       </c>
       <c r="F10" t="str">
-        <v>Status 200, trả về 2 chuyến đi</v>
+        <v>200 - trả về 2 chuyến đi</v>
       </c>
       <c r="G10" t="str">
         <v>PASS</v>
@@ -2226,10 +2221,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>/api/past-trips/detail/:id</v>
+        <v>GET</v>
       </c>
       <c r="C11" t="str">
-        <v>GET</v>
+        <v>/api/past-trips/detail/201</v>
       </c>
       <c r="D11" t="str">
         <v>id: 201</v>
@@ -2238,7 +2233,7 @@
         <v>200</v>
       </c>
       <c r="F11" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="G11" t="str">
         <v>PASS</v>
@@ -2249,10 +2244,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C12" t="str">
         <v>/api/payment/preview</v>
-      </c>
-      <c r="C12" t="str">
-        <v>GET</v>
       </c>
       <c r="D12" t="str">
         <v>Không có</v>
@@ -2261,7 +2256,7 @@
         <v>200</v>
       </c>
       <c r="F12" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="G12" t="str">
         <v>PASS</v>
@@ -2272,19 +2267,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
+        <v>POST</v>
+      </c>
+      <c r="C13" t="str">
         <v>/api/payment/process</v>
       </c>
-      <c r="C13" t="str">
-        <v>POST</v>
-      </c>
       <c r="D13" t="str">
-        <v>travelers: 2, total: 20</v>
+        <v>travelers: 2 / total: 20</v>
       </c>
       <c r="E13" t="str">
         <v>200</v>
       </c>
       <c r="F13" t="str">
-        <v>Status 200, success: true</v>
+        <v>200 - success: true</v>
       </c>
       <c r="G13" t="str">
         <v>PASS</v>
@@ -2295,10 +2290,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>/api/payment/process (thiếu body)</v>
+        <v>POST</v>
       </c>
       <c r="C14" t="str">
-        <v>POST</v>
+        <v>/api/payment/process (body rỗng)</v>
       </c>
       <c r="D14" t="str">
         <v>(trống)</v>
@@ -2307,7 +2302,7 @@
         <v>200</v>
       </c>
       <c r="F14" t="str">
-        <v>Status 200, dùng giá trị mặc định</v>
+        <v>200 - dùng giá trị mặc định</v>
       </c>
       <c r="G14" t="str">
         <v>PASS</v>
@@ -2318,10 +2313,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C15" t="str">
         <v>/api/profile</v>
-      </c>
-      <c r="C15" t="str">
-        <v>GET</v>
       </c>
       <c r="D15" t="str">
         <v>Không có</v>
@@ -2330,7 +2325,7 @@
         <v>200</v>
       </c>
       <c r="F15" t="str">
-        <v>Status 200, đúng dữ liệu</v>
+        <v>200 - đúng dữ liệu</v>
       </c>
       <c r="G15" t="str">
         <v>PASS</v>
@@ -2341,10 +2336,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C16" t="str">
         <v>/api/tourMore</v>
-      </c>
-      <c r="C16" t="str">
-        <v>GET</v>
       </c>
       <c r="D16" t="str">
         <v>Không có</v>
@@ -2353,7 +2348,7 @@
         <v>200</v>
       </c>
       <c r="F16" t="str">
-        <v>Status 200, trả về 8 tour</v>
+        <v>200 - trả về 8 tour</v>
       </c>
       <c r="G16" t="str">
         <v>PASS</v>
@@ -2364,10 +2359,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C17" t="str">
         <v>/api/tourMore?q=hanoi</v>
-      </c>
-      <c r="C17" t="str">
-        <v>GET</v>
       </c>
       <c r="D17" t="str">
         <v>q: hanoi</v>
@@ -2376,7 +2371,7 @@
         <v>200</v>
       </c>
       <c r="F17" t="str">
-        <v>Status 200, trả về tour có 'hanoi'</v>
+        <v>200 - tour có hanoi</v>
       </c>
       <c r="G17" t="str">
         <v>PASS</v>
@@ -2387,10 +2382,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>/api/tourMore/tours/:id/favorite</v>
+        <v>PATCH</v>
       </c>
       <c r="C18" t="str">
-        <v>PATCH</v>
+        <v>/api/tourMore/tours/1/favorite</v>
       </c>
       <c r="D18" t="str">
         <v>id: 1</v>
@@ -2399,7 +2394,7 @@
         <v>200</v>
       </c>
       <c r="F18" t="str">
-        <v>Status 200, favorite đảo ngược</v>
+        <v>200 - favorite đảo ngược</v>
       </c>
       <c r="G18" t="str">
         <v>PASS</v>
@@ -2410,10 +2405,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C19" t="str">
         <v>/api/wish-list</v>
-      </c>
-      <c r="C19" t="str">
-        <v>GET</v>
       </c>
       <c r="D19" t="str">
         <v>Không có</v>
@@ -2422,7 +2417,7 @@
         <v>200</v>
       </c>
       <c r="F19" t="str">
-        <v>Status 200, trả về 2 tour</v>
+        <v>200 - trả về 2 tour</v>
       </c>
       <c r="G19" t="str">
         <v>PASS</v>
@@ -2433,10 +2428,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>/api/wish-list/:id/like</v>
+        <v>PATCH</v>
       </c>
       <c r="C20" t="str">
-        <v>PATCH</v>
+        <v>/api/wish-list/301/like</v>
       </c>
       <c r="D20" t="str">
         <v>id: 301</v>
@@ -2445,7 +2440,7 @@
         <v>200</v>
       </c>
       <c r="F20" t="str">
-        <v>Status 200, liked đảo ngược</v>
+        <v>200 - liked đảo ngược</v>
       </c>
       <c r="G20" t="str">
         <v>PASS</v>
@@ -2456,10 +2451,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>/api/wish-list/:id</v>
+        <v>DELETE</v>
       </c>
       <c r="C21" t="str">
-        <v>DELETE</v>
+        <v>/api/wish-list/302</v>
       </c>
       <c r="D21" t="str">
         <v>id: 302</v>
@@ -2468,7 +2463,7 @@
         <v>200</v>
       </c>
       <c r="F21" t="str">
-        <v>Status 200, xóa thành công</v>
+        <v>200 - xóa thành công</v>
       </c>
       <c r="G21" t="str">
         <v>PASS</v>
@@ -2479,10 +2474,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>/api/wish-list/:id (not found)</v>
+        <v>DELETE</v>
       </c>
       <c r="C22" t="str">
-        <v>DELETE</v>
+        <v>/api/wish-list/999</v>
       </c>
       <c r="D22" t="str">
         <v>id: 999</v>
@@ -2491,7 +2486,7 @@
         <v>200</v>
       </c>
       <c r="F22" t="str">
-        <v>Status 404, trả về đúng message</v>
+        <v>404 - đúng message</v>
       </c>
       <c r="G22" t="str">
         <v>PASS</v>
@@ -2502,10 +2497,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C23" t="str">
         <v>/api/news</v>
-      </c>
-      <c r="C23" t="str">
-        <v>GET</v>
       </c>
       <c r="D23" t="str">
         <v>Không có</v>
@@ -2514,7 +2509,7 @@
         <v>200</v>
       </c>
       <c r="F23" t="str">
-        <v>Status 200, trả về 3 tin tức</v>
+        <v>200 - trả về 3 tin tức</v>
       </c>
       <c r="G23" t="str">
         <v>PASS</v>
@@ -2525,10 +2520,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C24" t="str">
         <v>/api/guides</v>
-      </c>
-      <c r="C24" t="str">
-        <v>GET</v>
       </c>
       <c r="D24" t="str">
         <v>Không có</v>
@@ -2537,7 +2532,7 @@
         <v>200</v>
       </c>
       <c r="F24" t="str">
-        <v>Status 200, trả về 2 hướng dẫn viên</v>
+        <v>200 - trả về 2 hướng dẫn viên</v>
       </c>
       <c r="G24" t="str">
         <v>PASS</v>

</xml_diff>